<commit_message>
Final human-edit CSBJ submission source data
</commit_message>
<xml_diff>
--- a/source_data/supplementary_tables/Supplementary_Table_5_software_environment.xlsx
+++ b/source_data/supplementary_tables/Supplementary_Table_5_software_environment.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supplement" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S5_Software_environment" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,12 +425,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="11" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="44" customWidth="1" min="3" max="3"/>
+    <col width="21" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -441,12 +442,17 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>role</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>version_source</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>version</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>source</t>
         </is>
       </c>
     </row>
@@ -458,12 +464,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Rscript (R) version 4.6.0 (2026-04-24)</t>
+          <t>Statistical analysis and visualization</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
           <t>Rscript --version</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>4.6.0 (2026-04-24)</t>
         </is>
       </c>
     </row>
@@ -475,97 +486,413 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>3.12.13</t>
+          <t>Analysis environment shell/version recorded during phase 0</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>/Users/baiqiu/.cache/codex-runtimes/codex-primary-runtime/dependencies/python/bin/python3</t>
+          <t>system python --version</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>3.9.6</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>OS</t>
+          <t>Python_packaging_QC</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>26.5.1</t>
+          <t>Document assembly, file QC and render helpers</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>sw_vers</t>
+          <t>bundled python --version</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>3.12.13</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ggplot2</t>
+          <t>Operating system</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>4.0.3</t>
+          <t>Analysis and packaging workstation</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>R packageVersion</t>
+          <t>sw_vers</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>macOS 26.5.1 (25F80)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>dplyr</t>
+          <t>ggplot2</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>1.2.1</t>
+          <t>Visualization</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>R packageVersion</t>
+          <t>R packageVersion("ggplot2")</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>4.0.3</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>readr</t>
+          <t>dplyr</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2.2.0</t>
+          <t>Data manipulation</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>R packageVersion</t>
+          <t>R packageVersion("dplyr")</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>1.2.1</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>readr</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Data import</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>R packageVersion("readr")</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>2.2.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>survival</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Cox proportional hazards models</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>R packageVersion("survival")</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>3.8.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>GEOquery</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>GEO access and metadata parsing</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>R packageVersion("GEOquery")</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>2.80.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Biobase</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>ExpressionSet handling</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>R packageVersion("Biobase")</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>2.72.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>limma</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Microarray utilities</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>R packageVersion("limma")</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>3.68.3</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>affy</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Affymetrix RMA processing</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>R packageVersion("affy")</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>1.90.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>preprocessCore</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Normalization support</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>R packageVersion("preprocessCore")</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>1.74.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>metafor</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Random-effects meta-analysis</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>R packageVersion("metafor")</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>5.0.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
           <t>openxlsx</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Supplementary workbook generation</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>R packageVersion("openxlsx")</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
         <is>
           <t>4.2.8.1</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>R packageVersion</t>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>patchwork</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Multi-panel figure assembly</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>R packageVersion("patchwork")</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>1.3.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>pheatmap</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Heatmap support</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>R packageVersion("pheatmap")</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>1.0.13</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>stringr</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>String handling</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>R packageVersion("stringr")</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>1.6.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>tidyr</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Data reshaping</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>R packageVersion("tidyr")</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>1.3.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>tibble</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Tabular data structures</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>R packageVersion("tibble")</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>3.3.1</t>
         </is>
       </c>
     </row>

</xml_diff>